<commit_message>
Option 3 excel save fixed
</commit_message>
<xml_diff>
--- a/queso.xlsx
+++ b/queso.xlsx
@@ -1,89 +1,56 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="promedio" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="promedio" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t xml:space="preserve">Matricula</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parcial 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parcial 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parcial 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Average</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Right to exam</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="4">
     <font>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -91,53 +58,110 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -314,78 +338,101 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.5390625" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="8.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.02"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="9.14"/>
+    <col width="10.86" customWidth="1" style="3" min="1" max="1"/>
+    <col width="8.710000000000001" customWidth="1" style="3" min="2" max="2"/>
+    <col width="8.31" customWidth="1" style="3" min="3" max="5"/>
+    <col width="10.57" customWidth="1" style="3" min="6" max="6"/>
+    <col width="17.02" customWidth="1" style="3" min="7" max="7"/>
+    <col width="9.140000000000001" customWidth="1" style="3" min="16384" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
+    <row r="1" ht="15" customHeight="1" s="4">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Matricula</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Parcial 1</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Parcial 2</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Parcial 3</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Right to exam</t>
+        </is>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+    <row r="2" ht="15" customHeight="1" s="4">
+      <c r="A2" s="5" t="n"/>
+      <c r="B2" s="5" t="n"/>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="5" t="n"/>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>has right</t>
+        </is>
+      </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+    <row r="3" ht="15" customHeight="1" s="4">
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>has right</t>
+        </is>
+      </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+    <row r="4" ht="15" customHeight="1" s="4">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>has right</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clean up + Some fixes
Added a .gitignore (used to not merge local changes to main)
</commit_message>
<xml_diff>
--- a/queso.xlsx
+++ b/queso.xlsx
@@ -1,70 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/471dfabb4741d0d0/Desktop/PROGR^J ESCU/python/Python-Grading-System/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_D8F10C661210B7E50121B7B73FA1A2D1946B6A28" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58E36ACE-C5A7-4D28-9C26-2F072A6EA113}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="promedio" sheetId="1" r:id="rId1"/>
+    <sheet name="promedio" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>Matricula</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Parcial 1</t>
-  </si>
-  <si>
-    <t>Parcial 2</t>
-  </si>
-  <si>
-    <t>Parcial 3</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
-  <si>
-    <t>Right to exam</t>
-  </si>
-  <si>
-    <t>394468</t>
-  </si>
-  <si>
-    <t>Josue Caleb Escobedo Herrera</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -83,27 +46,86 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -282,77 +304,113 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" customWidth="1"/>
-    <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="8.33203125" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="16384" max="16384" width="9.109375" customWidth="1"/>
+    <col width="10.88671875" customWidth="1" min="1" max="1"/>
+    <col width="25.88671875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="8.33203125" customWidth="1" min="3" max="5"/>
+    <col width="10.5546875" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="9.109375" customWidth="1" min="16384" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Matricula</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Parcial 1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Parcial 2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Parcial 3</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Right to exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>394569</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Eric Gallo Gardea</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
         <v>6</v>
       </c>
+      <c r="D2" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
     </row>
-    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>394468</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Josue Caleb Escobedo Herrera</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
     </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2">
-        <v>8</v>
-      </c>
-      <c r="D3" s="2">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2">
-        <v>8</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="1" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>